<commit_message>
outlier detection before flux calculations and attempt to deal with midnight samples
</commit_message>
<xml_diff>
--- a/data/Nutrients/Life Budget.xlsx
+++ b/data/Nutrients/Life Budget.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/keanurochette/Desktop/Git Hub Repository/MOBEAST/data/Nutrients/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96DB2A72-5485-DB4D-BBE5-BE1E71CB506D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E53B2B40-D4CA-174C-BC63-65D3C930361C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17300" activeTab="2" xr2:uid="{C0D20522-729A-9E49-BB3A-00A52D58EA3A}"/>
+    <workbookView xWindow="1100" yWindow="660" windowWidth="28040" windowHeight="17280" activeTab="1" xr2:uid="{C0D20522-729A-9E49-BB3A-00A52D58EA3A}"/>
   </bookViews>
   <sheets>
     <sheet name="2026 Template" sheetId="3" r:id="rId1"/>
-    <sheet name="September 2026" sheetId="2" r:id="rId2"/>
-    <sheet name="October 2026" sheetId="4" r:id="rId3"/>
+    <sheet name="September 2025" sheetId="2" r:id="rId2"/>
+    <sheet name="October 2025" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>